<commit_message>
결과 파일 업데이트 2026-08-29 06:25
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260829.xlsx
+++ b/results/andar_할인율모니터링_20260829.xlsx
@@ -979,7 +979,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3,488</t>
+          <t>3,489</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3,488</t>
+          <t>3,489</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10,011</t>
+          <t>10,012</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>345</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>345</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>343</t>
+          <t>345</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1327,37 +1327,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9620&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16649&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EMTBG-12</t>
+          <t>EPTBG-02</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>데일리 쇼퍼백</t>
+          <t>서밋 유틸리티 백팩</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>89,000</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>1,384</t>
+          <t>97</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1369,37 +1369,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16649&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9620&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EPTBG-02</t>
+          <t>EMTBG-12</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>서밋 유틸리티 백팩</t>
+          <t>데일리 쇼퍼백</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>89,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>1,384</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>407</t>
+          <t>408</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>714</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2,306</t>
+          <t>2,309</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1579,79 +1579,79 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15144&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EJFST-02</t>
+          <t>EOTBO-01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>릴렉스 요가링</t>
+          <t>액티브 스포츠 보틀 (650ml)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>3,900</t>
+          <t>15,000</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>6,544</t>
+          <t>216</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15144&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EOTBO-01</t>
+          <t>EOTBG-21</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>액티브 스포츠 보틀 (650ml)</t>
+          <t>데일리 라운드백</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>15,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>100</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1663,42 +1663,42 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EOTBG-21</t>
+          <t>EJFST-02</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>데일리 라운드백</t>
+          <t>릴렉스 요가링</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>3,900</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>6,545</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>273</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1831,84 +1831,84 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12318&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17414&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ENTBG-13</t>
+          <t>EPTBG-01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>데일리 스퀘어백</t>
+          <t>에어플라이 프리런 러닝 벨트</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>27,000</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>421</t>
+          <t>53</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17414&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12318&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EPTBG-01</t>
+          <t>ENTBG-13</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>에어플라이 프리런 러닝 벨트</t>
+          <t>데일리 스퀘어백</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>27,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>421</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1999,84 +1999,84 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13852&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EOTBG-10</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>에어플라이 투웨이 프리런 백 3.0</t>
+          <t>라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>1,124</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13852&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>EOTBG-10</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>라이트 러닝 베스트</t>
+          <t>에어플라이 투웨이 프리런 백 3.0</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>1,124</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>3.0</t>
         </is>
       </c>
     </row>
@@ -2167,42 +2167,42 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EOTBG-05</t>
+          <t>ENTSO-02</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>메쉬 포켓 비치백</t>
+          <t>안다르 제트플라이 (우먼즈)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>95,000</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>61%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>1,032</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ENTSO-02</t>
+          <t>ENTSO-12</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>1,031</t>
+          <t>1,032</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2251,42 +2251,42 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14059&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ENTSO-12</t>
+          <t>EOTBG-05</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (우먼즈)</t>
+          <t>메쉬 포켓 비치백</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>95,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>61%</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>1,031</t>
+          <t>41</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>351</t>
+          <t>352</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>687</t>
+          <t>688</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>56</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2755,42 +2755,42 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8726&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EMTSC-03</t>
+          <t>EOTSC-15</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>논슬립 서포트 풀 토삭스 (HOLE)</t>
+          <t>논슬립 퍼포먼스 풀 토삭스</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>4,806</t>
+          <t>143</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>609</t>
+          <t>611</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2881,42 +2881,42 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8726&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EOTSC-15</t>
+          <t>EMTSC-03</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 풀 토삭스</t>
+          <t>논슬립 서포트 풀 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>4,806</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>240</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3007,37 +3007,37 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EPTSC-04</t>
+          <t>EOTSV-03</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>필라테스 토삭스</t>
+          <t>서포트 허리 보호대</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>170</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3091,42 +3091,42 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EOTSV-03</t>
+          <t>EPTSC-04</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>서포트 허리 보호대</t>
+          <t>필라테스 토삭스</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>90</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -3175,84 +3175,84 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EMTSV-06</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
+          <t>에어쿨링 손목 보호대</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>657</t>
+          <t>1,079</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EMTSV-06</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>에어쿨링 손목 보호대</t>
+          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>1,079</t>
+          <t>658</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -3301,84 +3301,84 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ENTSC-20</t>
+          <t>EOTGL-01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>시그니처 로고 크루 삭스</t>
+          <t>짐 글러브 2.0</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>21,000</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>558</t>
+          <t>282</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EOTGL-01</t>
+          <t>ENTSC-20</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>짐 글러브 2.0</t>
+          <t>시그니처 로고 크루 삭스</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>21,000</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>280</t>
+          <t>559</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -3427,27 +3427,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 풀 토삭스</t>
+          <t>컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3457,91 +3457,91 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>338</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EOTSC-13</t>
+          <t>EKPMB-01</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>테이핑 테크 러닝 삭스</t>
+          <t>릴렉스 웨이트볼 0.5kg</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>682</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EKPMB-01</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>릴렉스 웨이트볼 0.5kg</t>
+          <t>맨즈 논슬립 풀 토삭스</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>682</t>
+          <t>97</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3553,163 +3553,163 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16650&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11962&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EPTCP-02</t>
+          <t>ENTMT-01</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>시그니처 로고 나일론 볼캡</t>
+          <t>레스트 인 마블 요가매트 (4mm)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>263</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EOTSC-13</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>컴프레션 러닝 니삭스</t>
+          <t>테이핑 테크 러닝 삭스</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>338</t>
+          <t>268</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11962&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16650&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ENTMT-01</t>
+          <t>EPTCP-02</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>레스트 인 마블 요가매트 (4mm)</t>
+          <t>시그니처 로고 나일론 볼캡</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>263</t>
+          <t>49</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EPTFB-02</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>퍼포먼스 심리스 손목밴드</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>504</t>
+          <t>250</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3721,42 +3721,42 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>EOTGL-04</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>논슬립 스킨 요기 글러브</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>504</t>
+          <t>178</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>1,572</t>
+          <t>1,573</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>1,572</t>
+          <t>1,573</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3877,7 +3877,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>1,572</t>
+          <t>1,573</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3889,79 +3889,79 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EOTGL-04</t>
+          <t>EMTRB-01</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>논슬립 스킨 요기 글러브</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>178</t>
+          <t>1,360</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EPTFB-02</t>
+          <t>EMTRB-02</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>퍼포먼스 심리스 손목밴드</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
+          <t>8,900</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
           <t>6,900</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>5,900</t>
-        </is>
-      </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>1,360</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3973,79 +3973,79 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EKPMB-02</t>
+          <t>EMTRB-03</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>릴렉스 미니 짐볼</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>1,219</t>
+          <t>1,360</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EMTRB-01</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>1,360</t>
+          <t>504</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4057,37 +4057,37 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EMTRB-02</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>1,360</t>
+          <t>504</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4099,42 +4099,42 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EMTRB-03</t>
+          <t>EKPMB-02</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>릴렉스 미니 짐볼</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1,360</t>
+          <t>1,219</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
@@ -4183,37 +4183,37 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17415&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EPTSC-01</t>
+          <t>ENTMK-01</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>쿨 메쉬 서포트 러닝 삭스</t>
+          <t>UV 프로텍션 맨즈 골프 마스크</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>15,000</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>1,530</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4225,42 +4225,42 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11027&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>ENTSC-08</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>맨즈 라이트 러닝 베스트</t>
+          <t>[5 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>85,000</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>59%</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>810</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -4309,84 +4309,84 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ENTMK-01</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>UV 프로텍션 맨즈 골프 마스크</t>
+          <t>[1&amp;1] 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>15,000</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>1,529</t>
+          <t>701</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>ENTFB-01</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
+          <t>에어쿨링 라인 스크런치</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>17,800</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>3,015</t>
+          <t>742</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4398,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4435,37 +4435,37 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 발목 보호대</t>
+          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>17,800</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>3,015</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4477,79 +4477,79 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11027&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ENTSC-08</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[5 SET] 에어컴피 크루 삭스</t>
+          <t>맨즈 라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>85,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>59%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>810</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ENTFB-01</t>
+          <t>EMTSC-01</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>에어쿨링 라인 스크런치</t>
+          <t>링글 크루 삭스</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>741</t>
+          <t>1,317</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4561,27 +4561,27 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EMTSC-01</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>링글 크루 삭스</t>
+          <t>논슬립 퍼포먼스 크루삭스</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4591,49 +4591,49 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>1,317</t>
+          <t>660</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
+          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>41,800</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>35,600</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>556</t>
+          <t>592</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4645,79 +4645,79 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 크루삭스</t>
+          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>660</t>
+          <t>556</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EOTSC-01</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
+          <t>프레시 필드 니삭스</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>41,800</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>35,600</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>592</t>
+          <t>292</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4729,37 +4729,37 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>296</t>
+          <t>688</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4813,37 +4813,37 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>하이 서포트 무릎 보호대</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
+          <t>23,800</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
           <t>14,900</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>10,900</t>
-        </is>
-      </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>687</t>
+          <t>296</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -4855,79 +4855,79 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 팔토시</t>
+          <t>논슬립 스킨 하프 토삭스</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>104</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EKPRB-04</t>
+          <t>ENTSC-12</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
+          <t>논슬립 퍼포먼스 토삭스</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>467</t>
+          <t>4,134</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -4939,121 +4939,121 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EKPRB-04</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>논슬립 스킨 하프 토삭스</t>
+          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>467</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EPTSC-05</t>
+          <t>EPTSC-02</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>필라테스 앵클 삭스</t>
+          <t>하이 쿠션 테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>86</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ENTSC-12</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 토삭스</t>
+          <t>[1&amp;1] 3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>4,133</t>
+          <t>543</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -5065,84 +5065,84 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16640&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>EPTBG-05</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>서포트 발목 보호대</t>
+          <t>안다르 시그니처 로고 에코백</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EPTSC-02</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>하이 쿠션 테이핑 러닝 삭스</t>
+          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>643</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5191,37 +5191,37 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EPTSC-05</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
+          <t>필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
+          <t>13,900</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
           <t>10,900</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>7,900</t>
-        </is>
-      </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>32</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -5233,79 +5233,79 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>ENTSC-07</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>[3 SET] 에어컴피 크루 삭스</t>
+          <t>서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>51,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>701</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17522&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>ENTSC-07</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 필라테스 삭스</t>
+          <t>[3 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>51,000</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>18,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>556</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EPTSC-08</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5359,17 +5359,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17522&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EPTSC-08</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
+          <t>[1&amp;1] 맨즈 필라테스 삭스</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -5379,59 +5379,59 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>18,900</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>32%</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>논슬립 스킨 토삭스</t>
+          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>588</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -5443,79 +5443,79 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
+          <t>논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>85</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EKPRB-05</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>릴렉스 4레벨 힙 밴드</t>
+          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>525</t>
+          <t>153</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5527,37 +5527,37 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17857&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>EKPRB-05</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>[1&amp;1] 데일리 루즈 삭스</t>
+          <t>릴렉스 4레벨 힙 밴드</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>525</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -5569,79 +5569,79 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17857&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ENTET-02</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 2kg</t>
+          <t>[1&amp;1] 데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17415&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EOTET-01</t>
+          <t>EPTSC-01</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>소프트 뱀부 롱 타월</t>
+          <t>쿨 메쉬 서포트 러닝 삭스</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>46%</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>114</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5653,37 +5653,37 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>EOTSC-10</t>
+          <t>EOTET-01</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>시그니처 로고 맨즈 크루 삭스</t>
+          <t>소프트 뱀부 롱 타월</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>233</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5695,32 +5695,32 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>EOTGL-02</t>
+          <t>EOTSC-10</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>히트 런 글러브</t>
+          <t>시그니처 로고 맨즈 크루 삭스</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5779,37 +5779,37 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16033&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EOTMK-02</t>
+          <t>EOTSC-04</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>소프텐션 넥마스크</t>
+          <t>올데이 수피마 스니커즈 삭스</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>4,500</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>423</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -5821,79 +5821,79 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>EOTSC-04</t>
+          <t>ENTET-02</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>올데이 수피마 스니커즈 삭스</t>
+          <t>릴렉스 소프트 웨이트바 2kg</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>4,500</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>423</t>
+          <t>76</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTGL-02</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>3D 쿨링 팔토시</t>
+          <t>히트 런 글러브</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>543</t>
+          <t>212</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -5905,269 +5905,269 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9612&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16033&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EMTSC-28</t>
+          <t>EOTMK-02</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>[1&amp;1] 리브드 셔링 루즈 삭스</t>
+          <t>소프텐션 넥마스크</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>157</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 1kg</t>
+          <t>3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>592</t>
+          <t>543</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9612&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>EMTSV-03</t>
+          <t>EMTSC-28</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>서포트 무릎 보호대</t>
+          <t>[1&amp;1] 리브드 셔링 루즈 삭스</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>1,981</t>
+          <t>393</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>EOTCP-03</t>
+          <t>EOTSC-05</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>쿨 라운드 볼캡</t>
+          <t>올데이 수피마 앵클 삭스</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>4,900</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>468</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>EOTSC-05</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>올데이 수피마 앵클 삭스</t>
+          <t>릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>4,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>468</t>
+          <t>592</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16640&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EPTBG-05</t>
+          <t>EMTSC-27</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>안다르 시그니처 로고 에코백</t>
+          <t>올라운드 오버 니삭스</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>292</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EMTSC-27</t>
+          <t>EMTSV-03</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>올라운드 오버 니삭스</t>
+          <t>서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -6177,22 +6177,22 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>1,981</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
@@ -6241,27 +6241,27 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>EOTSC-01</t>
+          <t>EOTCP-03</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>프레시 필드 니삭스</t>
+          <t>쿨 라운드 볼캡</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -6271,7 +6271,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -6325,37 +6325,37 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16036&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EOTCP-06</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>[1&amp;1] 레그 워머</t>
+          <t>소프트 니트 버킷햇</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>52</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -6372,7 +6372,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -6409,37 +6409,37 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16036&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EOTCP-06</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>소프트 니트 버킷햇</t>
+          <t>[1&amp;1] 레그 워머</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>230</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -6493,17 +6493,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 앵클 삭스</t>
+          <t>서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -6513,39 +6513,39 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>588</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>서포트 팔꿈치 보호대</t>
+          <t>맨즈 필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -6555,22 +6555,22 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>308</t>
+          <t>309</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -6661,153 +6661,153 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EOTMU-01</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>스트링 패딩 넥워머</t>
+          <t>데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>27</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>EPTSC-08</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>데일리 루즈 삭스</t>
+          <t>맨즈 필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EPTSC-08</t>
+          <t>EMTSC-29</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 크루 삭스</t>
+          <t>니트 루즈 삭스</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>513</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9993&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13831&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>EMTSC-29</t>
+          <t>EOTCP-02</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>니트 루즈 삭스</t>
+          <t>데님 로고 볼캡</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -6817,7 +6817,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>513</t>
+          <t>26</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -6829,27 +6829,27 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11725&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12480&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>ENTFB-04</t>
+          <t>ENTSC-24</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>더블 링글 손목밴드</t>
+          <t>웜 슬릿 레그 워머</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>4,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>4,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -6859,39 +6859,39 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>297</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12480&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>ENTSC-24</t>
+          <t>EOTSC-11</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>웜 슬릿 레그 워머</t>
+          <t>웜 레그 롱 워머</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -6901,39 +6901,39 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>297</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11725&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>EOTSC-11</t>
+          <t>ENTFB-04</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>웜 레그 롱 워머</t>
+          <t>더블 링글 손목밴드</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>4,900</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>4,900</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6943,49 +6943,49 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>433</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>ENTMU-01</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>소프트 니트 머플러</t>
+          <t>[1&amp;1] 램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>17,900</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>472</t>
+          <t>817</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -6997,42 +6997,42 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10191&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16045&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EOTMU-01</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>[1&amp;1] 램스울 크루 삭스</t>
+          <t>스트링 패딩 넥워머</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>17,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>816</t>
+          <t>46</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -7333,27 +7333,27 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13831&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12793&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>EOTCP-02</t>
+          <t>ENTMU-01</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>데님 로고 볼캡</t>
+          <t>소프트 니트 머플러</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -7363,7 +7363,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>472</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>555</t>
+          <t>556</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">

</xml_diff>